<commit_message>
feat: unificacion de modulos, actualizacion de dependencias, spec relativo y plantillas
</commit_message>
<xml_diff>
--- a/plantillas/plantilla_notificacion.xlsx
+++ b/plantillas/plantilla_notificacion.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jose.diarma\Desktop\Aplicacion_offline\App_Informes_Offline\plantillas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jose.diarma\Desktop\Macrolima\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -101,16 +101,16 @@
     <t>II)   Oficio N° xxx-2026-MINEDU/VMGI-PRONABEC-DIBEC</t>
   </si>
   <si>
-    <t>DIEGO CARBAJAL CCORAHUA</t>
-  </si>
-  <si>
-    <t>diegodacc864@gmail.com</t>
-  </si>
-  <si>
-    <t>60692-2026</t>
-  </si>
-  <si>
-    <t>I) Informe N° 6757-2026-MINEDU/VMGI-PRONABEC-DIBEC-SUS</t>
+    <t>PERICO DE LOS PALOTES</t>
+  </si>
+  <si>
+    <t>12345-2026</t>
+  </si>
+  <si>
+    <t>poltergeist@gmail.com</t>
+  </si>
+  <si>
+    <t>I) Informe N° 1234-2026-MINEDU/VMGI-PRONABEC-DIBEC-SUS</t>
   </si>
 </sst>
 </file>
@@ -424,6 +424,123 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
@@ -436,30 +553,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -486,99 +579,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -921,37 +921,37 @@
       <c r="C1" s="1"/>
     </row>
     <row r="2" spans="1:19" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="35"/>
-      <c r="L2" s="35"/>
-      <c r="M2" s="34"/>
-      <c r="N2" s="34"/>
-      <c r="O2" s="34"/>
-      <c r="P2" s="34"/>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="36"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="15"/>
     </row>
     <row r="3" spans="1:19" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="37" t="s">
+      <c r="B3" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="38"/>
-      <c r="D3" s="39"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="18"/>
       <c r="E3" s="4" t="s">
         <v>3</v>
       </c>
@@ -970,19 +970,19 @@
       <c r="J3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="K3" s="40" t="s">
+      <c r="K3" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="L3" s="41"/>
+      <c r="L3" s="20"/>
       <c r="M3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="N3" s="42" t="s">
+      <c r="N3" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="O3" s="43"/>
-      <c r="P3" s="43"/>
-      <c r="Q3" s="44"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
+      <c r="Q3" s="23"/>
       <c r="R3" s="3" t="s">
         <v>12</v>
       </c>
@@ -991,98 +991,100 @@
       </c>
     </row>
     <row r="4" spans="1:19" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="21">
+      <c r="A4" s="24">
         <v>1</v>
       </c>
-      <c r="B4" s="45" t="s">
+      <c r="B4" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="40"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="24">
+        <v>12345678</v>
+      </c>
+      <c r="F4" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="58" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="61" t="s">
+        <v>16</v>
+      </c>
+      <c r="K4" s="54" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="58"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="21">
-        <v>78969598</v>
-      </c>
-      <c r="F4" s="46" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" s="24" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" s="27" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" s="30" t="s">
-        <v>16</v>
-      </c>
-      <c r="K4" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="L4" s="16"/>
-      <c r="M4" s="49" t="s">
+      <c r="L4" s="41"/>
+      <c r="M4" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="N4" s="61" t="s">
+      <c r="N4" s="48" t="s">
         <v>24</v>
       </c>
-      <c r="O4" s="62"/>
-      <c r="P4" s="62"/>
-      <c r="Q4" s="63"/>
-      <c r="R4" s="52" t="s">
+      <c r="O4" s="49"/>
+      <c r="P4" s="49"/>
+      <c r="Q4" s="50"/>
+      <c r="R4" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="S4" s="55" t="s">
+      <c r="S4" s="36" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:19" s="2" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="22"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="59"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="47"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="31"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="50"/>
+      <c r="A5" s="25"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="59"/>
+      <c r="J5" s="62"/>
+      <c r="K5" s="42"/>
+      <c r="L5" s="44"/>
+      <c r="M5" s="31"/>
       <c r="N5" s="9" t="s">
         <v>20</v>
       </c>
       <c r="O5" s="8"/>
       <c r="P5" s="10"/>
       <c r="Q5" s="11"/>
-      <c r="R5" s="53"/>
-      <c r="S5" s="56"/>
+      <c r="R5" s="34"/>
+      <c r="S5" s="37"/>
     </row>
     <row r="6" spans="1:19" s="2" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="23"/>
-      <c r="B6" s="19"/>
-      <c r="C6" s="60"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="48"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="32"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="20"/>
-      <c r="M6" s="51"/>
-      <c r="N6" s="12"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="14"/>
-      <c r="R6" s="54"/>
-      <c r="S6" s="57"/>
+      <c r="A6" s="26"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="57"/>
+      <c r="I6" s="60"/>
+      <c r="J6" s="63"/>
+      <c r="K6" s="45"/>
+      <c r="L6" s="47"/>
+      <c r="M6" s="32"/>
+      <c r="N6" s="51"/>
+      <c r="O6" s="52"/>
+      <c r="P6" s="52"/>
+      <c r="Q6" s="53"/>
+      <c r="R6" s="35"/>
+      <c r="S6" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="I4:I6"/>
+    <mergeCell ref="J4:J6"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="K3:L3"/>
@@ -1099,8 +1101,6 @@
     <mergeCell ref="K4:L6"/>
     <mergeCell ref="G4:G6"/>
     <mergeCell ref="H4:H6"/>
-    <mergeCell ref="I4:I6"/>
-    <mergeCell ref="J4:J6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="K4" r:id="rId1"/>

</xml_diff>